<commit_message>
Code with screenshot capture class and method
</commit_message>
<xml_diff>
--- a/ConfigurationFiles/ExcelFiles/Loginpasswords.xlsx
+++ b/ConfigurationFiles/ExcelFiles/Loginpasswords.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sivaguruvaithy\eclipse-workspace\OrangeHRM\ConfigurationFiles\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA33C825-5FA6-4B3F-9241-C803F8041F45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{479CB1AF-FF65-42E0-A078-7277B57038EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{116C6692-C2E2-4F86-B54F-790ABB78C0AC}"/>
+    <workbookView xWindow="5760" yWindow="0" windowWidth="17280" windowHeight="8880" xr2:uid="{116C6692-C2E2-4F86-B54F-790ABB78C0AC}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginPageCredentials" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>userName</t>
   </si>
@@ -46,30 +46,6 @@
   </si>
   <si>
     <t>passWord</t>
-  </si>
-  <si>
-    <t>admin12</t>
-  </si>
-  <si>
-    <t>Admino</t>
-  </si>
-  <si>
-    <t>sivaguru</t>
-  </si>
-  <si>
-    <t>SivaGuru</t>
-  </si>
-  <si>
-    <t>marisurya</t>
-  </si>
-  <si>
-    <t>MariSurya</t>
-  </si>
-  <si>
-    <t>vijaykumar</t>
-  </si>
-  <si>
-    <t>Vijaykumar</t>
   </si>
 </sst>
 </file>
@@ -430,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{080B608A-EEBC-467E-8876-0009F09F7755}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.44140625" customWidth="1"/>
@@ -453,46 +429,6 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" t="s">
-        <v>11</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>